<commit_message>
[DEV] updates to incorproate print statements in pin_temp output, also save in params for later use
</commit_message>
<xml_diff>
--- a/examples/watts_exec_LTMR_pin_temp_output.xlsx
+++ b/examples/watts_exec_LTMR_pin_temp_output.xlsx
@@ -491,16 +491,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>39042313</v>
+        <v>39121205</v>
       </c>
       <c r="D2" t="n">
-        <v>39042313</v>
+        <v>39121205</v>
       </c>
       <c r="E2" t="n">
-        <v>4069468</v>
+        <v>4284463</v>
       </c>
       <c r="F2" t="n">
-        <v>4069468</v>
+        <v>4284463</v>
       </c>
       <c r="G2" t="n">
         <v>51</v>
@@ -525,16 +525,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>79600</v>
+        <v>77117</v>
       </c>
       <c r="D3" t="n">
-        <v>79600</v>
+        <v>77117</v>
       </c>
       <c r="E3" t="n">
-        <v>12440</v>
+        <v>11696</v>
       </c>
       <c r="F3" t="n">
-        <v>12440</v>
+        <v>11696</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>74609</v>
+        <v>73616</v>
       </c>
       <c r="D4" t="n">
-        <v>74609</v>
+        <v>73616</v>
       </c>
       <c r="E4" t="n">
-        <v>12207</v>
+        <v>10012</v>
       </c>
       <c r="F4" t="n">
-        <v>12207</v>
+        <v>10012</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -593,22 +593,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>28155528</v>
+        <v>27811055</v>
       </c>
       <c r="D5" t="n">
-        <v>28155528</v>
+        <v>27811055</v>
       </c>
       <c r="E5" t="n">
-        <v>3717502</v>
+        <v>3584577</v>
       </c>
       <c r="F5" t="n">
-        <v>3717502</v>
+        <v>3584577</v>
       </c>
       <c r="G5" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H5" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I5" t="n">
         <v>4</v>
@@ -627,16 +627,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5050198</v>
+        <v>5041133</v>
       </c>
       <c r="D6" t="n">
-        <v>5050198</v>
+        <v>5041133</v>
       </c>
       <c r="E6" t="n">
-        <v>1231559</v>
+        <v>1003007</v>
       </c>
       <c r="F6" t="n">
-        <v>1231559</v>
+        <v>1003007</v>
       </c>
       <c r="G6" t="n">
         <v>6</v>
@@ -661,22 +661,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5682376</v>
+        <v>6118282</v>
       </c>
       <c r="D7" t="n">
-        <v>5682376</v>
+        <v>6118282</v>
       </c>
       <c r="E7" t="n">
-        <v>1113184</v>
+        <v>1353579</v>
       </c>
       <c r="F7" t="n">
-        <v>1113184</v>
+        <v>1353579</v>
       </c>
       <c r="G7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I7" t="n">
         <v>1</v>
@@ -695,28 +695,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>111897500</v>
+        <v>110341826</v>
       </c>
       <c r="D8" t="n">
-        <v>45105880</v>
+        <v>43949474</v>
       </c>
       <c r="E8" t="n">
-        <v>15858405</v>
+        <v>18165276</v>
       </c>
       <c r="F8" t="n">
-        <v>9404888</v>
+        <v>10611728</v>
       </c>
       <c r="G8" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H8" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I8" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="J8" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -729,28 +729,28 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>16008174</v>
+        <v>15644659</v>
       </c>
       <c r="D9" t="n">
-        <v>3703468</v>
+        <v>3602989</v>
       </c>
       <c r="E9" t="n">
-        <v>6904398</v>
+        <v>8906055</v>
       </c>
       <c r="F9" t="n">
-        <v>1240214</v>
+        <v>1574594</v>
       </c>
       <c r="G9" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H9" t="n">
         <v>4</v>
       </c>
       <c r="I9" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -763,16 +763,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>200563</v>
+        <v>204872</v>
       </c>
       <c r="D10" t="n">
-        <v>115256</v>
+        <v>117732</v>
       </c>
       <c r="E10" t="n">
-        <v>21561</v>
+        <v>20820</v>
       </c>
       <c r="F10" t="n">
-        <v>12390</v>
+        <v>11964</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -797,16 +797,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>116817</v>
+        <v>119117</v>
       </c>
       <c r="D11" t="n">
-        <v>67130</v>
+        <v>68452</v>
       </c>
       <c r="E11" t="n">
-        <v>18214</v>
+        <v>18181</v>
       </c>
       <c r="F11" t="n">
-        <v>10467</v>
+        <v>10448</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -831,16 +831,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>69279</v>
+        <v>70614</v>
       </c>
       <c r="D12" t="n">
-        <v>39812</v>
+        <v>40579</v>
       </c>
       <c r="E12" t="n">
-        <v>10561</v>
+        <v>10324</v>
       </c>
       <c r="F12" t="n">
-        <v>6069</v>
+        <v>5932</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -865,16 +865,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>14466</v>
+        <v>15140</v>
       </c>
       <c r="D13" t="n">
-        <v>8313</v>
+        <v>8700</v>
       </c>
       <c r="E13" t="n">
-        <v>2331</v>
+        <v>2427</v>
       </c>
       <c r="F13" t="n">
-        <v>1339</v>
+        <v>1395</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -899,16 +899,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1842742</v>
+        <v>1747719</v>
       </c>
       <c r="D14" t="n">
-        <v>1058951</v>
+        <v>1004345</v>
       </c>
       <c r="E14" t="n">
-        <v>422136</v>
+        <v>417056</v>
       </c>
       <c r="F14" t="n">
-        <v>242585</v>
+        <v>239666</v>
       </c>
       <c r="G14" t="n">
         <v>2</v>
@@ -933,16 +933,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>198089</v>
+        <v>191588</v>
       </c>
       <c r="D15" t="n">
-        <v>113834</v>
+        <v>110098</v>
       </c>
       <c r="E15" t="n">
-        <v>28589</v>
+        <v>30638</v>
       </c>
       <c r="F15" t="n">
-        <v>16429</v>
+        <v>17606</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -967,16 +967,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>151221</v>
+        <v>155943</v>
       </c>
       <c r="D16" t="n">
-        <v>86901</v>
+        <v>89614</v>
       </c>
       <c r="E16" t="n">
-        <v>23652</v>
+        <v>24287</v>
       </c>
       <c r="F16" t="n">
-        <v>13592</v>
+        <v>13956</v>
       </c>
       <c r="G16" t="n">
         <v>0</v>
@@ -1001,16 +1001,16 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>161540</v>
+        <v>158380</v>
       </c>
       <c r="D17" t="n">
-        <v>92830</v>
+        <v>91015</v>
       </c>
       <c r="E17" t="n">
-        <v>24298</v>
+        <v>23853</v>
       </c>
       <c r="F17" t="n">
-        <v>13963</v>
+        <v>13707</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -1035,16 +1035,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1157584</v>
+        <v>1086520</v>
       </c>
       <c r="D18" t="n">
-        <v>665218</v>
+        <v>624380</v>
       </c>
       <c r="E18" t="n">
-        <v>409219</v>
+        <v>409001</v>
       </c>
       <c r="F18" t="n">
-        <v>235162</v>
+        <v>235036</v>
       </c>
       <c r="G18" t="n">
         <v>1</v>
@@ -1069,16 +1069,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>174306</v>
+        <v>155285</v>
       </c>
       <c r="D19" t="n">
-        <v>100166</v>
+        <v>89236</v>
       </c>
       <c r="E19" t="n">
-        <v>93069</v>
+        <v>72817</v>
       </c>
       <c r="F19" t="n">
-        <v>53483</v>
+        <v>41845</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -1103,16 +1103,16 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>76561</v>
+        <v>75693</v>
       </c>
       <c r="D20" t="n">
-        <v>43997</v>
+        <v>43498</v>
       </c>
       <c r="E20" t="n">
-        <v>5485</v>
+        <v>5259</v>
       </c>
       <c r="F20" t="n">
-        <v>3152</v>
+        <v>3022</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
@@ -1137,16 +1137,16 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>50987</v>
+        <v>50020</v>
       </c>
       <c r="D21" t="n">
-        <v>29300</v>
+        <v>28744</v>
       </c>
       <c r="E21" t="n">
-        <v>5019</v>
+        <v>4596</v>
       </c>
       <c r="F21" t="n">
-        <v>2884</v>
+        <v>2641</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -1171,16 +1171,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>15581</v>
+        <v>15626</v>
       </c>
       <c r="D22" t="n">
-        <v>8953</v>
+        <v>8979</v>
       </c>
       <c r="E22" t="n">
-        <v>2588</v>
+        <v>2494</v>
       </c>
       <c r="F22" t="n">
-        <v>1487</v>
+        <v>1433</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -1205,16 +1205,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>12542</v>
+        <v>12559</v>
       </c>
       <c r="D23" t="n">
-        <v>7207</v>
+        <v>7217</v>
       </c>
       <c r="E23" t="n">
-        <v>1804</v>
+        <v>1987</v>
       </c>
       <c r="F23" t="n">
-        <v>1036</v>
+        <v>1142</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -1239,16 +1239,16 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>22864</v>
+        <v>21835</v>
       </c>
       <c r="D24" t="n">
-        <v>13139</v>
+        <v>12547</v>
       </c>
       <c r="E24" t="n">
-        <v>3564</v>
+        <v>3385</v>
       </c>
       <c r="F24" t="n">
-        <v>2048</v>
+        <v>1945</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
@@ -1273,16 +1273,16 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>25573</v>
+        <v>25673</v>
       </c>
       <c r="D25" t="n">
-        <v>14696</v>
+        <v>14753</v>
       </c>
       <c r="E25" t="n">
-        <v>2404</v>
+        <v>2405</v>
       </c>
       <c r="F25" t="n">
-        <v>1381</v>
+        <v>1382</v>
       </c>
       <c r="G25" t="n">
         <v>0</v>
@@ -1307,16 +1307,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>7859</v>
+        <v>7957</v>
       </c>
       <c r="D26" t="n">
-        <v>4516</v>
+        <v>4573</v>
       </c>
       <c r="E26" t="n">
-        <v>1249</v>
+        <v>1132</v>
       </c>
       <c r="F26" t="n">
-        <v>717</v>
+        <v>651</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
@@ -1341,16 +1341,16 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>6260</v>
+        <v>6314</v>
       </c>
       <c r="D27" t="n">
-        <v>3597</v>
+        <v>3628</v>
       </c>
       <c r="E27" t="n">
-        <v>1013</v>
+        <v>949</v>
       </c>
       <c r="F27" t="n">
-        <v>582</v>
+        <v>545</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
@@ -1375,16 +1375,16 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>11454</v>
+        <v>11400</v>
       </c>
       <c r="D28" t="n">
-        <v>6582</v>
+        <v>6551</v>
       </c>
       <c r="E28" t="n">
-        <v>1879</v>
+        <v>1782</v>
       </c>
       <c r="F28" t="n">
-        <v>1079</v>
+        <v>1024</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
@@ -1409,28 +1409,28 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>13847495</v>
+        <v>13575590</v>
       </c>
       <c r="D29" t="n">
-        <v>2461811</v>
+        <v>2413977</v>
       </c>
       <c r="E29" t="n">
-        <v>6895649</v>
+        <v>8935364</v>
       </c>
       <c r="F29" t="n">
-        <v>1218357</v>
+        <v>1578931</v>
       </c>
       <c r="G29" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H29" t="n">
         <v>3</v>
       </c>
       <c r="I29" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -1443,28 +1443,28 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>13810133</v>
+        <v>13537691</v>
       </c>
       <c r="D30" t="n">
-        <v>2440340</v>
+        <v>2392198</v>
       </c>
       <c r="E30" t="n">
-        <v>6896026</v>
+        <v>8935380</v>
       </c>
       <c r="F30" t="n">
-        <v>1218572</v>
+        <v>1578939</v>
       </c>
       <c r="G30" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H30" t="n">
         <v>3</v>
       </c>
       <c r="I30" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
@@ -1477,28 +1477,28 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>13810133</v>
+        <v>13537691</v>
       </c>
       <c r="D31" t="n">
-        <v>2440340</v>
+        <v>2392198</v>
       </c>
       <c r="E31" t="n">
-        <v>6896026</v>
+        <v>8935380</v>
       </c>
       <c r="F31" t="n">
-        <v>1218572</v>
+        <v>1578939</v>
       </c>
       <c r="G31" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H31" t="n">
         <v>3</v>
       </c>
       <c r="I31" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
@@ -1511,16 +1511,16 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>37362</v>
+        <v>37898</v>
       </c>
       <c r="D32" t="n">
-        <v>21470</v>
+        <v>21778</v>
       </c>
       <c r="E32" t="n">
-        <v>3673</v>
+        <v>3166</v>
       </c>
       <c r="F32" t="n">
-        <v>2110</v>
+        <v>1819</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
@@ -1545,16 +1545,16 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>37362</v>
+        <v>37898</v>
       </c>
       <c r="D33" t="n">
-        <v>21470</v>
+        <v>21778</v>
       </c>
       <c r="E33" t="n">
-        <v>3673</v>
+        <v>3166</v>
       </c>
       <c r="F33" t="n">
-        <v>2110</v>
+        <v>1819</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
@@ -1579,16 +1579,16 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>6352</v>
+        <v>6393</v>
       </c>
       <c r="D34" t="n">
-        <v>3650</v>
+        <v>3673</v>
       </c>
       <c r="E34" t="n">
-        <v>938</v>
+        <v>889</v>
       </c>
       <c r="F34" t="n">
-        <v>539</v>
+        <v>511</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
@@ -1613,16 +1613,16 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>18501</v>
+        <v>18801</v>
       </c>
       <c r="D35" t="n">
-        <v>10632</v>
+        <v>10804</v>
       </c>
       <c r="E35" t="n">
-        <v>3117</v>
+        <v>2724</v>
       </c>
       <c r="F35" t="n">
-        <v>1791</v>
+        <v>1565</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -1647,16 +1647,16 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>12508</v>
+        <v>12703</v>
       </c>
       <c r="D36" t="n">
-        <v>7188</v>
+        <v>7300</v>
       </c>
       <c r="E36" t="n">
-        <v>1933</v>
+        <v>1865</v>
       </c>
       <c r="F36" t="n">
-        <v>1110</v>
+        <v>1072</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
@@ -1681,16 +1681,16 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>40811</v>
+        <v>40783</v>
       </c>
       <c r="D37" t="n">
-        <v>23452</v>
+        <v>23436</v>
       </c>
       <c r="E37" t="n">
-        <v>3654</v>
+        <v>4091</v>
       </c>
       <c r="F37" t="n">
-        <v>2100</v>
+        <v>2351</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
@@ -1715,16 +1715,16 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>40811</v>
+        <v>40783</v>
       </c>
       <c r="D38" t="n">
-        <v>23452</v>
+        <v>23436</v>
       </c>
       <c r="E38" t="n">
-        <v>3654</v>
+        <v>4091</v>
       </c>
       <c r="F38" t="n">
-        <v>2100</v>
+        <v>2351</v>
       </c>
       <c r="G38" t="n">
         <v>0</v>
@@ -1749,16 +1749,16 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>15811</v>
+        <v>15689</v>
       </c>
       <c r="D39" t="n">
-        <v>9086</v>
+        <v>9016</v>
       </c>
       <c r="E39" t="n">
-        <v>2567</v>
+        <v>2641</v>
       </c>
       <c r="F39" t="n">
-        <v>1475</v>
+        <v>1517</v>
       </c>
       <c r="G39" t="n">
         <v>0</v>
@@ -1783,16 +1783,16 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>12354</v>
+        <v>12308</v>
       </c>
       <c r="D40" t="n">
-        <v>7099</v>
+        <v>7073</v>
       </c>
       <c r="E40" t="n">
-        <v>1889</v>
+        <v>1879</v>
       </c>
       <c r="F40" t="n">
-        <v>1085</v>
+        <v>1079</v>
       </c>
       <c r="G40" t="n">
         <v>0</v>
@@ -1817,16 +1817,16 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>12645</v>
+        <v>12785</v>
       </c>
       <c r="D41" t="n">
-        <v>7266</v>
+        <v>7347</v>
       </c>
       <c r="E41" t="n">
-        <v>1928</v>
+        <v>2393</v>
       </c>
       <c r="F41" t="n">
-        <v>1108</v>
+        <v>1375</v>
       </c>
       <c r="G41" t="n">
         <v>0</v>
@@ -1851,22 +1851,22 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>58809948</v>
+        <v>59209200</v>
       </c>
       <c r="D42" t="n">
-        <v>15069287</v>
+        <v>15132222</v>
       </c>
       <c r="E42" t="n">
-        <v>6152471</v>
+        <v>6528590</v>
       </c>
       <c r="F42" t="n">
-        <v>1295391</v>
+        <v>1358509</v>
       </c>
       <c r="G42" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H42" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I42" t="n">
         <v>8</v>
@@ -1885,16 +1885,16 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>40075242</v>
+        <v>40642182</v>
       </c>
       <c r="D43" t="n">
-        <v>7891477</v>
+        <v>7993465</v>
       </c>
       <c r="E43" t="n">
-        <v>5602176</v>
+        <v>6084482</v>
       </c>
       <c r="F43" t="n">
-        <v>1004088</v>
+        <v>1126098</v>
       </c>
       <c r="G43" t="n">
         <v>53</v>
@@ -1903,7 +1903,7 @@
         <v>10</v>
       </c>
       <c r="I43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J43" t="n">
         <v>1</v>
@@ -1919,16 +1919,16 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>11411576</v>
+        <v>11397429</v>
       </c>
       <c r="D44" t="n">
-        <v>2945105</v>
+        <v>2941454</v>
       </c>
       <c r="E44" t="n">
-        <v>1322151</v>
+        <v>1313867</v>
       </c>
       <c r="F44" t="n">
-        <v>341221</v>
+        <v>339083</v>
       </c>
       <c r="G44" t="n">
         <v>15</v>
@@ -1953,16 +1953,16 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1370894</v>
+        <v>1370520</v>
       </c>
       <c r="D45" t="n">
-        <v>353801</v>
+        <v>353704</v>
       </c>
       <c r="E45" t="n">
-        <v>197648</v>
+        <v>236428</v>
       </c>
       <c r="F45" t="n">
-        <v>51009</v>
+        <v>61017</v>
       </c>
       <c r="G45" t="n">
         <v>1</v>
@@ -1987,16 +1987,16 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1023983</v>
+        <v>1043531</v>
       </c>
       <c r="D46" t="n">
-        <v>264270</v>
+        <v>269315</v>
       </c>
       <c r="E46" t="n">
-        <v>193479</v>
+        <v>171238</v>
       </c>
       <c r="F46" t="n">
-        <v>49933</v>
+        <v>44193</v>
       </c>
       <c r="G46" t="n">
         <v>1</v>
@@ -2021,16 +2021,16 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>9016698</v>
+        <v>8983377</v>
       </c>
       <c r="D47" t="n">
-        <v>2327034</v>
+        <v>2318434</v>
       </c>
       <c r="E47" t="n">
-        <v>1313795</v>
+        <v>1320010</v>
       </c>
       <c r="F47" t="n">
-        <v>339065</v>
+        <v>340669</v>
       </c>
       <c r="G47" t="n">
         <v>11</v>
@@ -2055,19 +2055,19 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>7620651</v>
+        <v>7447059</v>
       </c>
       <c r="D48" t="n">
-        <v>1227933</v>
+        <v>1200216</v>
       </c>
       <c r="E48" t="n">
-        <v>784053</v>
+        <v>826512</v>
       </c>
       <c r="F48" t="n">
-        <v>125491</v>
+        <v>132514</v>
       </c>
       <c r="G48" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H48" t="n">
         <v>1</v>
@@ -2089,19 +2089,19 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>7620651</v>
+        <v>7447059</v>
       </c>
       <c r="D49" t="n">
-        <v>1227933</v>
+        <v>1200216</v>
       </c>
       <c r="E49" t="n">
-        <v>784053</v>
+        <v>826512</v>
       </c>
       <c r="F49" t="n">
-        <v>125491</v>
+        <v>132514</v>
       </c>
       <c r="G49" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H49" t="n">
         <v>1</v>
@@ -2123,22 +2123,22 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>4802458</v>
+        <v>4653705</v>
       </c>
       <c r="D50" t="n">
-        <v>766235</v>
+        <v>742501</v>
       </c>
       <c r="E50" t="n">
-        <v>758764</v>
+        <v>756515</v>
       </c>
       <c r="F50" t="n">
-        <v>121061</v>
+        <v>120702</v>
       </c>
       <c r="G50" t="n">
         <v>6</v>
       </c>
       <c r="H50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I50" t="n">
         <v>1</v>
@@ -2157,16 +2157,16 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1099949</v>
+        <v>1097681</v>
       </c>
       <c r="D51" t="n">
-        <v>175497</v>
+        <v>175135</v>
       </c>
       <c r="E51" t="n">
-        <v>175619</v>
+        <v>169806</v>
       </c>
       <c r="F51" t="n">
-        <v>28020</v>
+        <v>27092</v>
       </c>
       <c r="G51" t="n">
         <v>1</v>
@@ -2191,16 +2191,16 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>658009</v>
+        <v>656563</v>
       </c>
       <c r="D52" t="n">
-        <v>116274</v>
+        <v>116018</v>
       </c>
       <c r="E52" t="n">
-        <v>95880</v>
+        <v>104269</v>
       </c>
       <c r="F52" t="n">
-        <v>16942</v>
+        <v>18425</v>
       </c>
       <c r="G52" t="n">
         <v>0</v>
@@ -2225,16 +2225,16 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>44603</v>
+        <v>44857</v>
       </c>
       <c r="D53" t="n">
-        <v>7881</v>
+        <v>7926</v>
       </c>
       <c r="E53" t="n">
-        <v>7165</v>
+        <v>6631</v>
       </c>
       <c r="F53" t="n">
-        <v>1266</v>
+        <v>1171</v>
       </c>
       <c r="G53" t="n">
         <v>0</v>
@@ -2259,16 +2259,16 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1015630</v>
+        <v>994252</v>
       </c>
       <c r="D54" t="n">
-        <v>162044</v>
+        <v>158633</v>
       </c>
       <c r="E54" t="n">
-        <v>151222</v>
+        <v>151225</v>
       </c>
       <c r="F54" t="n">
-        <v>24127</v>
+        <v>24128</v>
       </c>
       <c r="G54" t="n">
         <v>1</v>
@@ -2293,22 +2293,22 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>21043013</v>
+        <v>21797692</v>
       </c>
       <c r="D55" t="n">
-        <v>3718437</v>
+        <v>3851794</v>
       </c>
       <c r="E55" t="n">
-        <v>5591440</v>
+        <v>5749466</v>
       </c>
       <c r="F55" t="n">
-        <v>988043</v>
+        <v>1015968</v>
       </c>
       <c r="G55" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H55" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I55" t="n">
         <v>7</v>
@@ -2327,16 +2327,16 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>10418</v>
+        <v>10707</v>
       </c>
       <c r="D56" t="n">
-        <v>1841</v>
+        <v>1892</v>
       </c>
       <c r="E56" t="n">
-        <v>1815</v>
+        <v>2092</v>
       </c>
       <c r="F56" t="n">
-        <v>320</v>
+        <v>369</v>
       </c>
       <c r="G56" t="n">
         <v>0</v>
@@ -2361,16 +2361,16 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>-2347</v>
+        <v>-2397</v>
       </c>
       <c r="D57" t="n">
-        <v>-414</v>
+        <v>-423</v>
       </c>
       <c r="E57" t="n">
-        <v>336</v>
+        <v>449</v>
       </c>
       <c r="F57" t="n">
-        <v>59</v>
+        <v>79</v>
       </c>
       <c r="G57" t="n">
         <v>0</v>
@@ -2395,16 +2395,16 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>12765</v>
+        <v>13105</v>
       </c>
       <c r="D58" t="n">
-        <v>2255</v>
+        <v>2315</v>
       </c>
       <c r="E58" t="n">
-        <v>1831</v>
+        <v>2060</v>
       </c>
       <c r="F58" t="n">
-        <v>323</v>
+        <v>364</v>
       </c>
       <c r="G58" t="n">
         <v>0</v>
@@ -2429,19 +2429,19 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>20236994</v>
+        <v>20996211</v>
       </c>
       <c r="D59" t="n">
-        <v>3576008</v>
+        <v>3710167</v>
       </c>
       <c r="E59" t="n">
-        <v>5585229</v>
+        <v>5752594</v>
       </c>
       <c r="F59" t="n">
-        <v>986946</v>
+        <v>1016520</v>
       </c>
       <c r="G59" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H59" t="n">
         <v>4</v>
@@ -2463,19 +2463,19 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>20173689</v>
+        <v>20932513</v>
       </c>
       <c r="D60" t="n">
-        <v>3564822</v>
+        <v>3698911</v>
       </c>
       <c r="E60" t="n">
-        <v>5584223</v>
+        <v>5752597</v>
       </c>
       <c r="F60" t="n">
-        <v>986768</v>
+        <v>1016521</v>
       </c>
       <c r="G60" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H60" t="n">
         <v>4</v>
@@ -2497,16 +2497,16 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>63304</v>
+        <v>63697</v>
       </c>
       <c r="D61" t="n">
-        <v>11186</v>
+        <v>11255</v>
       </c>
       <c r="E61" t="n">
-        <v>12187</v>
+        <v>10482</v>
       </c>
       <c r="F61" t="n">
-        <v>2153</v>
+        <v>1852</v>
       </c>
       <c r="G61" t="n">
         <v>0</v>
@@ -2531,16 +2531,16 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>795601</v>
+        <v>790773</v>
       </c>
       <c r="D62" t="n">
-        <v>140587</v>
+        <v>139734</v>
       </c>
       <c r="E62" t="n">
-        <v>132619</v>
+        <v>122434</v>
       </c>
       <c r="F62" t="n">
-        <v>23434</v>
+        <v>21634</v>
       </c>
       <c r="G62" t="n">
         <v>1</v>
@@ -2565,19 +2565,19 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>6736044</v>
+        <v>6806631</v>
       </c>
       <c r="D63" t="n">
-        <v>5057568</v>
+        <v>5060620</v>
       </c>
       <c r="E63" t="n">
-        <v>888430</v>
+        <v>990546</v>
       </c>
       <c r="F63" t="n">
-        <v>717764</v>
+        <v>690581</v>
       </c>
       <c r="G63" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H63" t="n">
         <v>6</v>
@@ -2599,16 +2599,16 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1197778</v>
+        <v>1271848</v>
       </c>
       <c r="D64" t="n">
-        <v>211655</v>
+        <v>224743</v>
       </c>
       <c r="E64" t="n">
-        <v>635938</v>
+        <v>709170</v>
       </c>
       <c r="F64" t="n">
-        <v>112374</v>
+        <v>125314</v>
       </c>
       <c r="G64" t="n">
         <v>1</v>
@@ -2633,16 +2633,16 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1197778</v>
+        <v>1271848</v>
       </c>
       <c r="D65" t="n">
-        <v>211655</v>
+        <v>224743</v>
       </c>
       <c r="E65" t="n">
-        <v>635938</v>
+        <v>709170</v>
       </c>
       <c r="F65" t="n">
-        <v>112374</v>
+        <v>125314</v>
       </c>
       <c r="G65" t="n">
         <v>1</v>
@@ -2667,16 +2667,16 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>191242</v>
+        <v>191725</v>
       </c>
       <c r="D66" t="n">
-        <v>33793</v>
+        <v>33879</v>
       </c>
       <c r="E66" t="n">
-        <v>29609</v>
+        <v>28606</v>
       </c>
       <c r="F66" t="n">
-        <v>5232</v>
+        <v>5054</v>
       </c>
       <c r="G66" t="n">
         <v>0</v>
@@ -2701,16 +2701,16 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>649712</v>
+        <v>657190</v>
       </c>
       <c r="D67" t="n">
-        <v>114808</v>
+        <v>116129</v>
       </c>
       <c r="E67" t="n">
-        <v>83242</v>
+        <v>97387</v>
       </c>
       <c r="F67" t="n">
-        <v>14709</v>
+        <v>17209</v>
       </c>
       <c r="G67" t="n">
         <v>0</v>
@@ -2735,16 +2735,16 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>649712</v>
+        <v>657190</v>
       </c>
       <c r="D68" t="n">
-        <v>114808</v>
+        <v>116129</v>
       </c>
       <c r="E68" t="n">
-        <v>83242</v>
+        <v>97387</v>
       </c>
       <c r="F68" t="n">
-        <v>14709</v>
+        <v>17209</v>
       </c>
       <c r="G68" t="n">
         <v>0</v>
@@ -2769,16 +2769,16 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>4697311</v>
+        <v>4685867</v>
       </c>
       <c r="D69" t="n">
-        <v>4697311</v>
+        <v>4685867</v>
       </c>
       <c r="E69" t="n">
-        <v>729285</v>
+        <v>677261</v>
       </c>
       <c r="F69" t="n">
-        <v>729285</v>
+        <v>677261</v>
       </c>
       <c r="G69" t="n">
         <v>6</v>
@@ -2803,16 +2803,16 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1096766</v>
+        <v>1065101</v>
       </c>
       <c r="D70" t="n">
-        <v>193805</v>
+        <v>188210</v>
       </c>
       <c r="E70" t="n">
-        <v>124706</v>
+        <v>113845</v>
       </c>
       <c r="F70" t="n">
-        <v>22036</v>
+        <v>20117</v>
       </c>
       <c r="G70" t="n">
         <v>1</v>
@@ -2837,16 +2837,16 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1096766</v>
+        <v>1065101</v>
       </c>
       <c r="D71" t="n">
-        <v>193805</v>
+        <v>188210</v>
       </c>
       <c r="E71" t="n">
-        <v>124706</v>
+        <v>113845</v>
       </c>
       <c r="F71" t="n">
-        <v>22036</v>
+        <v>20117</v>
       </c>
       <c r="G71" t="n">
         <v>1</v>
@@ -2871,16 +2871,16 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>517615</v>
+        <v>512211</v>
       </c>
       <c r="D72" t="n">
-        <v>91466</v>
+        <v>90511</v>
       </c>
       <c r="E72" t="n">
-        <v>92565</v>
+        <v>77840</v>
       </c>
       <c r="F72" t="n">
-        <v>16356</v>
+        <v>13754</v>
       </c>
       <c r="G72" t="n">
         <v>0</v>
@@ -2905,16 +2905,16 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>579151</v>
+        <v>552890</v>
       </c>
       <c r="D73" t="n">
-        <v>102339</v>
+        <v>97699</v>
       </c>
       <c r="E73" t="n">
-        <v>91820</v>
+        <v>83269</v>
       </c>
       <c r="F73" t="n">
-        <v>16225</v>
+        <v>14714</v>
       </c>
       <c r="G73" t="n">
         <v>0</v>
@@ -2939,16 +2939,16 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>549200</v>
+        <v>548326</v>
       </c>
       <c r="D74" t="n">
-        <v>97047</v>
+        <v>96892</v>
       </c>
       <c r="E74" t="n">
-        <v>137951</v>
+        <v>111756</v>
       </c>
       <c r="F74" t="n">
-        <v>24376</v>
+        <v>19748</v>
       </c>
       <c r="G74" t="n">
         <v>0</v>
@@ -2973,16 +2973,16 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>10316809</v>
+        <v>10109781</v>
       </c>
       <c r="D75" t="n">
-        <v>1823047</v>
+        <v>1786464</v>
       </c>
       <c r="E75" t="n">
-        <v>2276792</v>
+        <v>2143242</v>
       </c>
       <c r="F75" t="n">
-        <v>402324</v>
+        <v>378724</v>
       </c>
       <c r="G75" t="n">
         <v>13</v>
@@ -2991,7 +2991,7 @@
         <v>2</v>
       </c>
       <c r="I75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J75" t="n">
         <v>0</v>
@@ -3007,16 +3007,16 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>35885</v>
+        <v>37177</v>
       </c>
       <c r="D76" t="n">
-        <v>6341</v>
+        <v>6569</v>
       </c>
       <c r="E76" t="n">
-        <v>7201</v>
+        <v>8724</v>
       </c>
       <c r="F76" t="n">
-        <v>1272</v>
+        <v>1541</v>
       </c>
       <c r="G76" t="n">
         <v>0</v>
@@ -3041,28 +3041,28 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>19751483</v>
+        <v>18715284</v>
       </c>
       <c r="D77" t="n">
-        <v>13414049</v>
+        <v>12692465</v>
       </c>
       <c r="E77" t="n">
-        <v>13224796</v>
+        <v>14238732</v>
       </c>
       <c r="F77" t="n">
-        <v>9352094</v>
+        <v>10106805</v>
       </c>
       <c r="G77" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H77" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I77" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J77" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="78">
@@ -3075,28 +3075,28 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>18566396</v>
+        <v>17558958</v>
       </c>
       <c r="D78" t="n">
-        <v>13204636</v>
+        <v>12488134</v>
       </c>
       <c r="E78" t="n">
-        <v>13125158</v>
+        <v>14202052</v>
       </c>
       <c r="F78" t="n">
-        <v>9334765</v>
+        <v>10100664</v>
       </c>
       <c r="G78" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H78" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I78" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J78" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="79">
@@ -3109,28 +3109,28 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>18566396</v>
+        <v>17558958</v>
       </c>
       <c r="D79" t="n">
-        <v>13204636</v>
+        <v>12488134</v>
       </c>
       <c r="E79" t="n">
-        <v>13125158</v>
+        <v>14202052</v>
       </c>
       <c r="F79" t="n">
-        <v>9334765</v>
+        <v>10100664</v>
       </c>
       <c r="G79" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H79" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I79" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J79" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="80">
@@ -3143,16 +3143,16 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1185087</v>
+        <v>1156326</v>
       </c>
       <c r="D80" t="n">
-        <v>209412</v>
+        <v>204330</v>
       </c>
       <c r="E80" t="n">
-        <v>254666</v>
+        <v>272595</v>
       </c>
       <c r="F80" t="n">
-        <v>45001</v>
+        <v>48169</v>
       </c>
       <c r="G80" t="n">
         <v>1</v>
@@ -3177,25 +3177,25 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>11072672</v>
+        <v>10523158</v>
       </c>
       <c r="D81" t="n">
-        <v>7875013</v>
+        <v>7484192</v>
       </c>
       <c r="E81" t="n">
-        <v>3939036</v>
+        <v>3532627</v>
       </c>
       <c r="F81" t="n">
-        <v>2801488</v>
+        <v>2512445</v>
       </c>
       <c r="G81" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H81" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I81" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J81" t="n">
         <v>3</v>
@@ -3211,16 +3211,16 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1072444</v>
+        <v>1070299</v>
       </c>
       <c r="D82" t="n">
-        <v>762734</v>
+        <v>761209</v>
       </c>
       <c r="E82" t="n">
-        <v>490859</v>
+        <v>679114</v>
       </c>
       <c r="F82" t="n">
-        <v>349105</v>
+        <v>482994</v>
       </c>
       <c r="G82" t="n">
         <v>1</v>
@@ -3245,16 +3245,16 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>803562</v>
+        <v>810587</v>
       </c>
       <c r="D83" t="n">
-        <v>571502</v>
+        <v>576499</v>
       </c>
       <c r="E83" t="n">
-        <v>422219</v>
+        <v>439274</v>
       </c>
       <c r="F83" t="n">
-        <v>300287</v>
+        <v>312416</v>
       </c>
       <c r="G83" t="n">
         <v>1</v>
@@ -3279,16 +3279,16 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>304420</v>
+        <v>304389</v>
       </c>
       <c r="D84" t="n">
-        <v>216507</v>
+        <v>216485</v>
       </c>
       <c r="E84" t="n">
-        <v>152152</v>
+        <v>180200</v>
       </c>
       <c r="F84" t="n">
-        <v>108212</v>
+        <v>128160</v>
       </c>
       <c r="G84" t="n">
         <v>0</v>
@@ -3313,16 +3313,16 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>836395</v>
+        <v>762015</v>
       </c>
       <c r="D85" t="n">
-        <v>594854</v>
+        <v>541954</v>
       </c>
       <c r="E85" t="n">
-        <v>489493</v>
+        <v>498421</v>
       </c>
       <c r="F85" t="n">
-        <v>348133</v>
+        <v>354482</v>
       </c>
       <c r="G85" t="n">
         <v>1</v>
@@ -3347,28 +3347,28 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>4662448</v>
+        <v>4379859</v>
       </c>
       <c r="D86" t="n">
-        <v>3315987</v>
+        <v>3115006</v>
       </c>
       <c r="E86" t="n">
-        <v>3529068</v>
+        <v>2632683</v>
       </c>
       <c r="F86" t="n">
-        <v>2509914</v>
+        <v>1872394</v>
       </c>
       <c r="G86" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H86" t="n">
         <v>4</v>
       </c>
       <c r="I86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="87">
@@ -3381,16 +3381,16 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>3393401</v>
+        <v>3196006</v>
       </c>
       <c r="D87" t="n">
-        <v>2413426</v>
+        <v>2273036</v>
       </c>
       <c r="E87" t="n">
-        <v>1794023</v>
+        <v>1763293</v>
       </c>
       <c r="F87" t="n">
-        <v>1275930</v>
+        <v>1254075</v>
       </c>
       <c r="G87" t="n">
         <v>4</v>
@@ -3415,16 +3415,16 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>4784107</v>
+        <v>4777485</v>
       </c>
       <c r="D88" t="n">
-        <v>4784107</v>
+        <v>4777485</v>
       </c>
       <c r="E88" t="n">
-        <v>1038371</v>
+        <v>918501</v>
       </c>
       <c r="F88" t="n">
-        <v>1038371</v>
+        <v>918501</v>
       </c>
       <c r="G88" t="n">
         <v>6</v>
@@ -3449,16 +3449,16 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2949220</v>
+        <v>2837569</v>
       </c>
       <c r="D89" t="n">
-        <v>2949220</v>
+        <v>2837569</v>
       </c>
       <c r="E89" t="n">
-        <v>524641</v>
+        <v>475680</v>
       </c>
       <c r="F89" t="n">
-        <v>524641</v>
+        <v>475680</v>
       </c>
       <c r="G89" t="n">
         <v>3</v>
@@ -3483,16 +3483,16 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>235041</v>
+        <v>243963</v>
       </c>
       <c r="D90" t="n">
-        <v>235041</v>
+        <v>243963</v>
       </c>
       <c r="E90" t="n">
-        <v>36984</v>
+        <v>36818</v>
       </c>
       <c r="F90" t="n">
-        <v>36984</v>
+        <v>36818</v>
       </c>
       <c r="G90" t="n">
         <v>0</v>
@@ -3517,16 +3517,16 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1599845</v>
+        <v>1695952</v>
       </c>
       <c r="D91" t="n">
-        <v>1599845</v>
+        <v>1695952</v>
       </c>
       <c r="E91" t="n">
-        <v>814152</v>
+        <v>795254</v>
       </c>
       <c r="F91" t="n">
-        <v>814152</v>
+        <v>795254</v>
       </c>
       <c r="G91" t="n">
         <v>2</v>
@@ -3551,16 +3551,16 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1471113</v>
+        <v>1472037</v>
       </c>
       <c r="D92" t="n">
-        <v>259955</v>
+        <v>260118</v>
       </c>
       <c r="E92" t="n">
-        <v>314992</v>
+        <v>344483</v>
       </c>
       <c r="F92" t="n">
-        <v>55661</v>
+        <v>60872</v>
       </c>
       <c r="G92" t="n">
         <v>1</v>
@@ -3585,16 +3585,16 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>13145877</v>
+        <v>12912496</v>
       </c>
       <c r="D93" t="n">
-        <v>5631474</v>
+        <v>5478573</v>
       </c>
       <c r="E93" t="n">
-        <v>1763820</v>
+        <v>2094535</v>
       </c>
       <c r="F93" t="n">
-        <v>835227</v>
+        <v>902362</v>
       </c>
       <c r="G93" t="n">
         <v>17</v>
@@ -3619,16 +3619,16 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>6183900</v>
+        <v>6118480</v>
       </c>
       <c r="D94" t="n">
-        <v>2104692</v>
+        <v>2055053</v>
       </c>
       <c r="E94" t="n">
-        <v>1033067</v>
+        <v>1159227</v>
       </c>
       <c r="F94" t="n">
-        <v>615462</v>
+        <v>668441</v>
       </c>
       <c r="G94" t="n">
         <v>8</v>
@@ -3653,16 +3653,16 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1732940</v>
+        <v>1699738</v>
       </c>
       <c r="D95" t="n">
-        <v>521859</v>
+        <v>496038</v>
       </c>
       <c r="E95" t="n">
-        <v>918362</v>
+        <v>1224753</v>
       </c>
       <c r="F95" t="n">
-        <v>245781</v>
+        <v>295236</v>
       </c>
       <c r="G95" t="n">
         <v>2</v>
@@ -3687,19 +3687,19 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>3019120</v>
+        <v>2865852</v>
       </c>
       <c r="D96" t="n">
-        <v>1734969</v>
+        <v>1646892</v>
       </c>
       <c r="E96" t="n">
-        <v>708137</v>
+        <v>644237</v>
       </c>
       <c r="F96" t="n">
-        <v>406938</v>
+        <v>370217</v>
       </c>
       <c r="G96" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H96" t="n">
         <v>2</v>
@@ -3721,16 +3721,16 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1002418</v>
+        <v>1009909</v>
       </c>
       <c r="D97" t="n">
-        <v>576050</v>
+        <v>580355</v>
       </c>
       <c r="E97" t="n">
-        <v>221234</v>
+        <v>240479</v>
       </c>
       <c r="F97" t="n">
-        <v>127134</v>
+        <v>138194</v>
       </c>
       <c r="G97" t="n">
         <v>1</v>
@@ -3755,16 +3755,16 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>720070</v>
+        <v>722677</v>
       </c>
       <c r="D98" t="n">
-        <v>413796</v>
+        <v>415294</v>
       </c>
       <c r="E98" t="n">
-        <v>168967</v>
+        <v>151950</v>
       </c>
       <c r="F98" t="n">
-        <v>97098</v>
+        <v>87319</v>
       </c>
       <c r="G98" t="n">
         <v>0</v>
@@ -3789,16 +3789,16 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>487428</v>
+        <v>495838</v>
       </c>
       <c r="D99" t="n">
-        <v>280105</v>
+        <v>284939</v>
       </c>
       <c r="E99" t="n">
-        <v>102927</v>
+        <v>109886</v>
       </c>
       <c r="F99" t="n">
-        <v>59148</v>
+        <v>63147</v>
       </c>
       <c r="G99" t="n">
         <v>0</v>
@@ -3823,16 +3823,16 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>345493</v>
+        <v>337069</v>
       </c>
       <c r="D100" t="n">
-        <v>345493</v>
+        <v>337069</v>
       </c>
       <c r="E100" t="n">
-        <v>70378</v>
+        <v>78059</v>
       </c>
       <c r="F100" t="n">
-        <v>70378</v>
+        <v>78059</v>
       </c>
       <c r="G100" t="n">
         <v>0</v>
@@ -3857,16 +3857,16 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>345493</v>
+        <v>337069</v>
       </c>
       <c r="D101" t="n">
-        <v>345493</v>
+        <v>337069</v>
       </c>
       <c r="E101" t="n">
-        <v>70378</v>
+        <v>78059</v>
       </c>
       <c r="F101" t="n">
-        <v>70378</v>
+        <v>78059</v>
       </c>
       <c r="G101" t="n">
         <v>0</v>
@@ -3891,16 +3891,16 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>2838056</v>
+        <v>2808393</v>
       </c>
       <c r="D102" t="n">
-        <v>1555546</v>
+        <v>1534163</v>
       </c>
       <c r="E102" t="n">
-        <v>309317</v>
+        <v>353444</v>
       </c>
       <c r="F102" t="n">
-        <v>185069</v>
+        <v>217503</v>
       </c>
       <c r="G102" t="n">
         <v>3</v>
@@ -3925,16 +3925,16 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>2838056</v>
+        <v>2808393</v>
       </c>
       <c r="D103" t="n">
-        <v>1555546</v>
+        <v>1534163</v>
       </c>
       <c r="E103" t="n">
-        <v>309317</v>
+        <v>353444</v>
       </c>
       <c r="F103" t="n">
-        <v>185069</v>
+        <v>217503</v>
       </c>
       <c r="G103" t="n">
         <v>3</v>
@@ -3959,28 +3959,28 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>7455450</v>
+        <v>7327941</v>
       </c>
       <c r="D104" t="n">
-        <v>3446051</v>
+        <v>3355042</v>
       </c>
       <c r="E104" t="n">
-        <v>563442</v>
+        <v>673122</v>
       </c>
       <c r="F104" t="n">
-        <v>327304</v>
+        <v>398924</v>
       </c>
       <c r="G104" t="n">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="H104" t="n">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="I104" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J104" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="105">
@@ -3993,22 +3993,22 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1386668</v>
+        <v>1337026</v>
       </c>
       <c r="D105" t="n">
-        <v>1386668</v>
+        <v>1337026</v>
       </c>
       <c r="E105" t="n">
-        <v>174573</v>
+        <v>170961</v>
       </c>
       <c r="F105" t="n">
-        <v>174573</v>
+        <v>170961</v>
       </c>
       <c r="G105" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H105" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I105" t="n">
         <v>3</v>
@@ -4027,22 +4027,22 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>371507</v>
+        <v>378099</v>
       </c>
       <c r="D106" t="n">
-        <v>371507</v>
+        <v>378099</v>
       </c>
       <c r="E106" t="n">
-        <v>59541</v>
+        <v>66408</v>
       </c>
       <c r="F106" t="n">
-        <v>59541</v>
+        <v>66408</v>
       </c>
       <c r="G106" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H106" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I106" t="n">
         <v>1</v>
@@ -4061,22 +4061,22 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1015160</v>
+        <v>958927</v>
       </c>
       <c r="D107" t="n">
-        <v>1015160</v>
+        <v>958927</v>
       </c>
       <c r="E107" t="n">
-        <v>154774</v>
+        <v>152543</v>
       </c>
       <c r="F107" t="n">
-        <v>154774</v>
+        <v>152543</v>
       </c>
       <c r="G107" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H107" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I107" t="n">
         <v>2</v>
@@ -4095,16 +4095,16 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>124581</v>
+        <v>123323</v>
       </c>
       <c r="D108" t="n">
-        <v>124581</v>
+        <v>123323</v>
       </c>
       <c r="E108" t="n">
-        <v>25965</v>
+        <v>26258</v>
       </c>
       <c r="F108" t="n">
-        <v>25965</v>
+        <v>26258</v>
       </c>
       <c r="G108" t="n">
         <v>2</v>
@@ -4129,28 +4129,28 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>5873399</v>
+        <v>5797483</v>
       </c>
       <c r="D109" t="n">
-        <v>1895330</v>
+        <v>1855726</v>
       </c>
       <c r="E109" t="n">
-        <v>537537</v>
+        <v>606107</v>
       </c>
       <c r="F109" t="n">
-        <v>288392</v>
+        <v>326185</v>
       </c>
       <c r="G109" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H109" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I109" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J109" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="110">
@@ -4163,16 +4163,16 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>173645</v>
+        <v>176960</v>
       </c>
       <c r="D110" t="n">
-        <v>44814</v>
+        <v>45669</v>
       </c>
       <c r="E110" t="n">
-        <v>32809</v>
+        <v>29038</v>
       </c>
       <c r="F110" t="n">
-        <v>8467</v>
+        <v>7494</v>
       </c>
       <c r="G110" t="n">
         <v>3</v>
@@ -4197,16 +4197,16 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1529033</v>
+        <v>1523383</v>
       </c>
       <c r="D111" t="n">
-        <v>394613</v>
+        <v>393155</v>
       </c>
       <c r="E111" t="n">
-        <v>222790</v>
+        <v>223844</v>
       </c>
       <c r="F111" t="n">
-        <v>57497</v>
+        <v>57769</v>
       </c>
       <c r="G111" t="n">
         <v>28</v>
@@ -4231,16 +4231,16 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>134916</v>
+        <v>134097</v>
       </c>
       <c r="D112" t="n">
-        <v>23840</v>
+        <v>23695</v>
       </c>
       <c r="E112" t="n">
-        <v>22489</v>
+        <v>20762</v>
       </c>
       <c r="F112" t="n">
-        <v>3974</v>
+        <v>3668</v>
       </c>
       <c r="G112" t="n">
         <v>2</v>
@@ -4265,16 +4265,16 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1766</v>
+        <v>1815</v>
       </c>
       <c r="D113" t="n">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="E113" t="n">
-        <v>307</v>
+        <v>354</v>
       </c>
       <c r="F113" t="n">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="G113" t="n">
         <v>0</v>
@@ -4299,19 +4299,19 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1292295</v>
+        <v>1262857</v>
       </c>
       <c r="D114" t="n">
-        <v>208230</v>
+        <v>203530</v>
       </c>
       <c r="E114" t="n">
-        <v>132958</v>
+        <v>140158</v>
       </c>
       <c r="F114" t="n">
-        <v>21280</v>
+        <v>22471</v>
       </c>
       <c r="G114" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H114" t="n">
         <v>3</v>
@@ -4333,25 +4333,25 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2741742</v>
+        <v>2698368</v>
       </c>
       <c r="D115" t="n">
-        <v>1223518</v>
+        <v>1189353</v>
       </c>
       <c r="E115" t="n">
-        <v>474859</v>
+        <v>539085</v>
       </c>
       <c r="F115" t="n">
-        <v>282325</v>
+        <v>317010</v>
       </c>
       <c r="G115" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H115" t="n">
         <v>22</v>
       </c>
       <c r="I115" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J115" t="n">
         <v>5</v>
@@ -4367,16 +4367,16 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>70800</v>
+        <v>70107</v>
       </c>
       <c r="D116" t="n">
-        <v>39470</v>
+        <v>38965</v>
       </c>
       <c r="E116" t="n">
-        <v>7707</v>
+        <v>8820</v>
       </c>
       <c r="F116" t="n">
-        <v>4708</v>
+        <v>5581</v>
       </c>
       <c r="G116" t="n">
         <v>1</v>
@@ -4401,16 +4401,16 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>874215</v>
+        <v>870153</v>
       </c>
       <c r="D117" t="n">
-        <v>874215</v>
+        <v>870153</v>
       </c>
       <c r="E117" t="n">
-        <v>178391</v>
+        <v>155450</v>
       </c>
       <c r="F117" t="n">
-        <v>178391</v>
+        <v>155450</v>
       </c>
       <c r="G117" t="n">
         <v>16</v>
@@ -4419,10 +4419,10 @@
         <v>16</v>
       </c>
       <c r="I117" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J117" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118">
@@ -4435,16 +4435,16 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1631</v>
+        <v>1693</v>
       </c>
       <c r="D118" t="n">
-        <v>1631</v>
+        <v>1693</v>
       </c>
       <c r="E118" t="n">
-        <v>267</v>
+        <v>297</v>
       </c>
       <c r="F118" t="n">
-        <v>267</v>
+        <v>297</v>
       </c>
       <c r="G118" t="n">
         <v>0</v>
@@ -4469,16 +4469,16 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>811279</v>
+        <v>810156</v>
       </c>
       <c r="D119" t="n">
-        <v>811279</v>
+        <v>810156</v>
       </c>
       <c r="E119" t="n">
-        <v>176084</v>
+        <v>155757</v>
       </c>
       <c r="F119" t="n">
-        <v>176084</v>
+        <v>155757</v>
       </c>
       <c r="G119" t="n">
         <v>15</v>
@@ -4487,10 +4487,10 @@
         <v>15</v>
       </c>
       <c r="I119" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J119" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120">
@@ -4503,16 +4503,16 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>61304</v>
+        <v>58304</v>
       </c>
       <c r="D120" t="n">
-        <v>61304</v>
+        <v>58304</v>
       </c>
       <c r="E120" t="n">
-        <v>10171</v>
+        <v>9513</v>
       </c>
       <c r="F120" t="n">
-        <v>10171</v>
+        <v>9513</v>
       </c>
       <c r="G120" t="n">
         <v>1</v>
@@ -4539,16 +4539,16 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>164431185</v>
+        <v>162712598</v>
       </c>
       <c r="D121" t="n">
-        <v>90125162</v>
+        <v>88886323</v>
       </c>
       <c r="E121" t="n">
-        <v>17921202</v>
+        <v>20477842</v>
       </c>
       <c r="F121" t="n">
-        <v>10722530</v>
+        <v>12601689</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
@@ -4583,16 +4583,16 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>26521</v>
+        <v>26243</v>
       </c>
       <c r="D122" t="n">
-        <v>14536</v>
+        <v>14336</v>
       </c>
       <c r="E122" t="n">
-        <v>2890</v>
+        <v>3302</v>
       </c>
       <c r="F122" t="n">
-        <v>1729</v>
+        <v>2032</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
@@ -4627,16 +4627,16 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>159647077</v>
+        <v>157935112</v>
       </c>
       <c r="D123" t="n">
-        <v>85341055</v>
+        <v>84108837</v>
       </c>
       <c r="E123" t="n">
-        <v>17994594</v>
+        <v>20329596</v>
       </c>
       <c r="F123" t="n">
-        <v>10753906</v>
+        <v>12453824</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
@@ -4671,16 +4671,16 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>25749</v>
+        <v>25473</v>
       </c>
       <c r="D124" t="n">
-        <v>13764</v>
+        <v>13565</v>
       </c>
       <c r="E124" t="n">
-        <v>2902</v>
+        <v>3278</v>
       </c>
       <c r="F124" t="n">
-        <v>1734</v>
+        <v>2008</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
@@ -4715,16 +4715,16 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>167269241</v>
+        <v>165520991</v>
       </c>
       <c r="D125" t="n">
-        <v>91680708</v>
+        <v>90420486</v>
       </c>
       <c r="E125" t="n">
-        <v>18230519</v>
+        <v>20831286</v>
       </c>
       <c r="F125" t="n">
-        <v>10907600</v>
+        <v>12819192</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
@@ -4759,16 +4759,16 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>26978</v>
+        <v>26696</v>
       </c>
       <c r="D126" t="n">
-        <v>14787</v>
+        <v>14583</v>
       </c>
       <c r="E126" t="n">
-        <v>2940</v>
+        <v>3359</v>
       </c>
       <c r="F126" t="n">
-        <v>1759</v>
+        <v>2067</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
@@ -4803,16 +4803,16 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>120034765</v>
+        <v>118780196</v>
       </c>
       <c r="D127" t="n">
-        <v>65791368</v>
+        <v>64887015</v>
       </c>
       <c r="E127" t="n">
-        <v>13082477</v>
+        <v>14948824</v>
       </c>
       <c r="F127" t="n">
-        <v>7827447</v>
+        <v>9199233</v>
       </c>
       <c r="G127" t="inlineStr">
         <is>
@@ -4847,16 +4847,16 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>19360</v>
+        <v>19158</v>
       </c>
       <c r="D128" t="n">
-        <v>10611</v>
+        <v>10465</v>
       </c>
       <c r="E128" t="n">
-        <v>2110</v>
+        <v>2411</v>
       </c>
       <c r="F128" t="n">
-        <v>1262</v>
+        <v>1483</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -4891,16 +4891,16 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>122872821</v>
+        <v>121588590</v>
       </c>
       <c r="D129" t="n">
-        <v>67346914</v>
+        <v>66421179</v>
       </c>
       <c r="E129" t="n">
-        <v>13391794</v>
+        <v>15302269</v>
       </c>
       <c r="F129" t="n">
-        <v>8012516</v>
+        <v>9416736</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
@@ -4935,16 +4935,16 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>19818</v>
+        <v>19611</v>
       </c>
       <c r="D130" t="n">
-        <v>10862</v>
+        <v>10713</v>
       </c>
       <c r="E130" t="n">
-        <v>2159</v>
+        <v>2468</v>
       </c>
       <c r="F130" t="n">
-        <v>1292</v>
+        <v>1518</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
@@ -4979,16 +4979,16 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>8329665</v>
+        <v>8198095</v>
       </c>
       <c r="D131" t="n">
-        <v>4320266</v>
+        <v>4225196</v>
       </c>
       <c r="E131" t="n">
-        <v>594378</v>
+        <v>710094</v>
       </c>
       <c r="F131" t="n">
-        <v>384359</v>
+        <v>452534</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
@@ -5023,16 +5023,16 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D132" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E132" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F132" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
@@ -5067,16 +5067,16 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="D133" t="n">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="E133" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F133" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
@@ -5111,16 +5111,16 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="D134" t="n">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E134" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="F134" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
@@ -5155,16 +5155,16 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D135" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E135" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F135" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
@@ -7306,7 +7306,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>[1.9536550591226562, 1.8679519000725917, 1.9026523110293394]</t>
+          <t>[1.9536550591226562, 1.8679519000725917, 1.9026523110293396]</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -7680,7 +7680,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>[1.3899464228403677, 1.357250310440318, 0.9416309033137141]</t>
+          <t>[1.3899464228403604, 1.3572503104403237, 0.9416309033136908]</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -7707,7 +7707,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>[1.3741950900711597, 1.3416440281071742, 0.929352547670816]</t>
+          <t>[1.3741950900711524, 1.34164402810718, 0.929352547670793]</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
@@ -12287,7 +12287,7 @@
         </is>
       </c>
       <c r="C271" t="n">
-        <v>1290.313509651437</v>
+        <v>1119.505019845636</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -12312,7 +12312,7 @@
         </is>
       </c>
       <c r="C272" t="n">
-        <v>1993.463509651437</v>
+        <v>1822.655019845636</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>

</xml_diff>